<commit_message>
Hi, I've added Bass Coast in the nest section, but not yet for threat data. However, I'm getting errors about the fate column when I import data (Row 2530). I've tried to trouble shoot but cant work out how to fix it.
</commit_message>
<xml_diff>
--- a/data/nest_issues_commented/BSC_nest_data_issues_220825.xlsx
+++ b/data/nest_issues_commented/BSC_nest_data_issues_220825.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t xml:space="preserve">season</t>
   </si>
@@ -111,31 +111,31 @@
     <t xml:space="preserve">issues</t>
   </si>
   <si>
-    <t xml:space="preserve">202122</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Point Lonsdale West of 4W</t>
-  </si>
-  <si>
-    <t xml:space="preserve">202122_Point Lonsdale 3W - 4W_4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06012022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23022022</t>
+    <t xml:space="preserve">201314</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8W Ocean Grove</t>
+  </si>
+  <si>
+    <t xml:space="preserve">201314_8W Ocean Grove_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22112013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26122013</t>
   </si>
   <si>
     <t xml:space="preserve">0</t>
   </si>
   <si>
-    <t xml:space="preserve">foredune/face</t>
+    <t xml:space="preserve">not specified</t>
   </si>
   <si>
     <t xml:space="preserve">Y</t>
   </si>
   <si>
-    <t xml:space="preserve">,</t>
+    <t xml:space="preserve">signaccess,signnest,ropefence</t>
   </si>
   <si>
     <t xml:space="preserve">1/3 adult size, fluffy</t>
@@ -144,55 +144,31 @@
     <t xml:space="preserve">MP</t>
   </si>
   <si>
+    <t xml:space="preserve">34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nest habitat is not beach, dune, foredune/face, or estuary/spit; </t>
+  </si>
+  <si>
+    <t xml:space="preserve">201011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13th Beach 29W-31W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">201011_13th Beach 29W - 31W_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03012011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01012011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
     <t xml:space="preserve">35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Management type is not sufficient for making levels; </t>
-  </si>
-  <si>
-    <t xml:space="preserve">201314</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8W Ocean Grove</t>
-  </si>
-  <si>
-    <t xml:space="preserve">201314_8W Ocean Grove_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22112013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26122013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">not specified</t>
-  </si>
-  <si>
-    <t xml:space="preserve">signaccess,signnest,ropefence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nest habitat is not beach, dune, foredune/face, estuary/spit, or rocks; </t>
-  </si>
-  <si>
-    <t xml:space="preserve">201011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13th Beach 29W-31W</t>
-  </si>
-  <si>
-    <t xml:space="preserve">201011_13th Beach 29W - 31W_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">03012011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01012011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N</t>
   </si>
   <si>
     <t xml:space="preserve">Pt Roadknight West Beach (96W)</t>
@@ -674,40 +650,40 @@
       <c r="K2"/>
       <c r="L2"/>
       <c r="M2" s="1" t="n">
-        <v>44618</v>
+        <v>41626</v>
       </c>
       <c r="N2" s="1" t="n">
-        <v>44580</v>
+        <v>41599</v>
       </c>
       <c r="O2" t="s">
         <v>41</v>
       </c>
       <c r="P2" s="1" t="n">
-        <v>44615</v>
+        <v>41634</v>
       </c>
       <c r="Q2" s="1" t="n">
-        <v>44580</v>
+        <v>41600</v>
       </c>
       <c r="R2" s="1" t="n">
-        <v>44615</v>
+        <v>41634</v>
       </c>
       <c r="S2" t="n">
-        <v>199</v>
+        <v>141</v>
       </c>
       <c r="T2" t="n">
-        <v>234</v>
+        <v>175</v>
       </c>
       <c r="U2" t="n">
-        <v>234</v>
+        <v>175</v>
       </c>
       <c r="V2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y2" t="n">
         <v>0</v>
@@ -718,9 +694,11 @@
       <c r="AA2" t="n">
         <v>0</v>
       </c>
-      <c r="AB2"/>
+      <c r="AB2" t="n">
+        <v>3</v>
+      </c>
       <c r="AC2" t="n">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="AD2" t="s">
         <v>42</v>
@@ -755,63 +733,63 @@
         <v>37</v>
       </c>
       <c r="H3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" t="s">
         <v>50</v>
       </c>
-      <c r="I3" t="s">
-        <v>39</v>
-      </c>
       <c r="J3" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="K3"/>
       <c r="L3"/>
       <c r="M3" s="1" t="n">
-        <v>41626</v>
+        <v>40547</v>
       </c>
       <c r="N3" s="1" t="n">
-        <v>41599</v>
+        <v>40509</v>
       </c>
       <c r="O3" t="s">
         <v>41</v>
       </c>
       <c r="P3" s="1" t="n">
-        <v>41634</v>
+        <v>40544</v>
       </c>
       <c r="Q3" s="1" t="n">
-        <v>41600</v>
+        <v>40509</v>
       </c>
       <c r="R3" s="1" t="n">
-        <v>41634</v>
+        <v>40544</v>
       </c>
       <c r="S3" t="n">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="T3" t="n">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="U3" t="n">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
         <v>1</v>
       </c>
-      <c r="W3" t="n">
-        <v>1</v>
-      </c>
-      <c r="X3" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>0</v>
-      </c>
       <c r="AB3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AC3" t="n">
         <v>244</v>
@@ -820,80 +798,80 @@
         <v>42</v>
       </c>
       <c r="AE3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AF3" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" t="s">
         <v>54</v>
       </c>
-      <c r="B4" t="s">
+      <c r="E4" t="s">
         <v>55</v>
       </c>
-      <c r="C4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" t="s">
-        <v>58</v>
-      </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G4" t="s">
         <v>37</v>
       </c>
       <c r="H4" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="I4" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J4" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="K4"/>
       <c r="L4"/>
       <c r="M4" s="1" t="n">
-        <v>40547</v>
+        <v>40480</v>
       </c>
       <c r="N4" s="1" t="n">
-        <v>40509</v>
+        <v>40442</v>
       </c>
       <c r="O4" t="s">
         <v>41</v>
       </c>
       <c r="P4" s="1" t="n">
-        <v>40544</v>
+        <v>40477</v>
       </c>
       <c r="Q4" s="1" t="n">
-        <v>40509</v>
+        <v>40452</v>
       </c>
       <c r="R4" s="1" t="n">
-        <v>40544</v>
+        <v>40477</v>
       </c>
       <c r="S4" t="n">
-        <v>146</v>
+        <v>89</v>
       </c>
       <c r="T4" t="n">
-        <v>181</v>
+        <v>114</v>
       </c>
       <c r="U4" t="n">
-        <v>181</v>
+        <v>114</v>
       </c>
       <c r="V4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y4" t="n">
         <v>0</v>
@@ -902,10 +880,10 @@
         <v>0</v>
       </c>
       <c r="AA4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AC4" t="n">
         <v>244</v>
@@ -914,104 +892,10 @@
         <v>42</v>
       </c>
       <c r="AE4" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="AF4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" t="s">
-        <v>60</v>
-      </c>
-      <c r="C5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D5" t="s">
-        <v>62</v>
-      </c>
-      <c r="E5" t="s">
-        <v>63</v>
-      </c>
-      <c r="F5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G5" t="s">
-        <v>37</v>
-      </c>
-      <c r="H5" t="s">
-        <v>50</v>
-      </c>
-      <c r="I5" t="s">
-        <v>39</v>
-      </c>
-      <c r="J5" t="s">
-        <v>51</v>
-      </c>
-      <c r="K5"/>
-      <c r="L5"/>
-      <c r="M5" s="1" t="n">
-        <v>40480</v>
-      </c>
-      <c r="N5" s="1" t="n">
-        <v>40442</v>
-      </c>
-      <c r="O5" t="s">
-        <v>41</v>
-      </c>
-      <c r="P5" s="1" t="n">
-        <v>40477</v>
-      </c>
-      <c r="Q5" s="1" t="n">
-        <v>40452</v>
-      </c>
-      <c r="R5" s="1" t="n">
-        <v>40477</v>
-      </c>
-      <c r="S5" t="n">
-        <v>89</v>
-      </c>
-      <c r="T5" t="n">
-        <v>114</v>
-      </c>
-      <c r="U5" t="n">
-        <v>114</v>
-      </c>
-      <c r="V5" t="n">
-        <v>1</v>
-      </c>
-      <c r="W5" t="n">
-        <v>1</v>
-      </c>
-      <c r="X5" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>244</v>
-      </c>
-      <c r="AD5" t="s">
-        <v>42</v>
-      </c>
-      <c r="AE5" t="s">
-        <v>64</v>
-      </c>
-      <c r="AF5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated all files and changed code to work out hatch dates to 28 days incubation length
</commit_message>
<xml_diff>
--- a/data/nest_issues_commented/BSC_nest_data_issues_220825.xlsx
+++ b/data/nest_issues_commented/BSC_nest_data_issues_220825.xlsx
@@ -156,34 +156,34 @@
     <t xml:space="preserve">13th Beach 29W-31W</t>
   </si>
   <si>
-    <t xml:space="preserve">201011_13th Beach 29W - 31W_1</t>
+    <t xml:space="preserve">201011_13th Beach 29W-31W_1</t>
   </si>
   <si>
     <t xml:space="preserve">03012011</t>
   </si>
   <si>
-    <t xml:space="preserve">01012011</t>
+    <t xml:space="preserve">08012011</t>
   </si>
   <si>
     <t xml:space="preserve">N</t>
   </si>
   <si>
-    <t xml:space="preserve">35</t>
+    <t xml:space="preserve">5</t>
   </si>
   <si>
     <t xml:space="preserve">Pt Roadknight West Beach (96W)</t>
   </si>
   <si>
-    <t xml:space="preserve">201011_Point Roadknight West (96W - 98W)_2</t>
+    <t xml:space="preserve">201011_Pt Roadknight West Beach (96W)_2</t>
   </si>
   <si>
     <t xml:space="preserve">01102010</t>
   </si>
   <si>
-    <t xml:space="preserve">26102010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">25</t>
+    <t xml:space="preserve">02112010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32</t>
   </si>
 </sst>
 </file>
@@ -747,28 +747,28 @@
         <v>40547</v>
       </c>
       <c r="N3" s="1" t="n">
-        <v>40509</v>
+        <v>40516</v>
       </c>
       <c r="O3" t="s">
         <v>41</v>
       </c>
       <c r="P3" s="1" t="n">
-        <v>40544</v>
+        <v>40551</v>
       </c>
       <c r="Q3" s="1" t="n">
-        <v>40509</v>
+        <v>40546</v>
       </c>
       <c r="R3" s="1" t="n">
-        <v>40544</v>
+        <v>40551</v>
       </c>
       <c r="S3" t="n">
-        <v>146</v>
+        <v>183</v>
       </c>
       <c r="T3" t="n">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="U3" t="n">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="V3" t="n">
         <v>0</v>
@@ -841,28 +841,28 @@
         <v>40480</v>
       </c>
       <c r="N4" s="1" t="n">
-        <v>40442</v>
+        <v>40449</v>
       </c>
       <c r="O4" t="s">
         <v>41</v>
       </c>
       <c r="P4" s="1" t="n">
-        <v>40477</v>
+        <v>40484</v>
       </c>
       <c r="Q4" s="1" t="n">
         <v>40452</v>
       </c>
       <c r="R4" s="1" t="n">
-        <v>40477</v>
+        <v>40484</v>
       </c>
       <c r="S4" t="n">
         <v>89</v>
       </c>
       <c r="T4" t="n">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="U4" t="n">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="V4" t="n">
         <v>1</v>

</xml_diff>